<commit_message>
feat: Enhance coverage heatmap with PAX skills toggle and add verification script
- Added a toggle to display only PAX-derived skills in the coverage heatmap.
- Updated the coverage data building logic to conditionally include PAX skills.
- Modified the coverage table rendering to reflect the selected skills.
- Introduced a new Python script `verify_intraday.py` to test the optimization of a specific date and check for PAX skills in the result.
- Updated relevant JavaScript files to support the new functionality.
</commit_message>
<xml_diff>
--- a/data/PAX Config.xlsx
+++ b/data/PAX Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9979a6a62ab1ab53/Coding/python_scripts/DAA-Project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="11_F25DC773A252ABDACC104835C91E41EE5ADE58E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90B59A00-2FA4-4ADF-9623-92A4615188D4}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="11_F25DC773A252ABDACC104835C91E41EE5ADE58E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B018ABF8-A393-4EA8-A3BC-9BCD2B090B89}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -119,6 +119,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -464,7 +468,7 @@
         <v>150</v>
       </c>
       <c r="F2">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="G2">
         <v>300</v>
@@ -485,7 +489,7 @@
         <v>150</v>
       </c>
       <c r="M2">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="N2">
         <v>300</v>

</xml_diff>

<commit_message>
feat: Enhance passenger capacity estimation and update UI for passenger metrics
</commit_message>
<xml_diff>
--- a/data/PAX Config.xlsx
+++ b/data/PAX Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9979a6a62ab1ab53/Coding/python_scripts/DAA-Project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_F25DC773A252ABDACC104835C91E41EE5ADE58E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B018ABF8-A393-4EA8-A3BC-9BCD2B090B89}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="11_F25DC773A252ABDACC104835C91E41EE5ADE58E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80D32420-5569-4008-A125-0852AD3C4042}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -453,7 +453,7 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="B2">
         <v>100</v>
@@ -474,7 +474,7 @@
         <v>300</v>
       </c>
       <c r="H2">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="I2">
         <v>100</v>

</xml_diff>

<commit_message>
Long term sorted with PAX forecast
</commit_message>
<xml_diff>
--- a/data/PAX Config.xlsx
+++ b/data/PAX Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9979a6a62ab1ab53/Coding/python_scripts/DAA-Project/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6070f6eab8483c11/Desktop/DAA/live/DAA-Project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="11_F25DC773A252ABDACC104835C91E41EE5ADE58E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80D32420-5569-4008-A125-0852AD3C4042}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="11_F25DC773A252ABDACC104835C91E41EE5ADE58E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{876FFA43-5221-40C9-AB91-598849D0A682}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,9 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -27,46 +30,46 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
-    <t>T1_checkin</t>
-  </si>
-  <si>
-    <t>T1_security</t>
-  </si>
-  <si>
-    <t>T1_cbp</t>
-  </si>
-  <si>
-    <t>T1_lounge</t>
-  </si>
-  <si>
-    <t>T1_boarding</t>
-  </si>
-  <si>
-    <t>T1_immigration</t>
-  </si>
-  <si>
-    <t>T1_baggage</t>
-  </si>
-  <si>
-    <t>T2_checkin</t>
-  </si>
-  <si>
-    <t>T2_security</t>
-  </si>
-  <si>
-    <t>T2_cbp</t>
-  </si>
-  <si>
-    <t>T2_lounge</t>
-  </si>
-  <si>
-    <t>T2_boarding</t>
-  </si>
-  <si>
-    <t>T2_immigration</t>
-  </si>
-  <si>
-    <t>T2_baggage</t>
+    <t>T1_Checkin</t>
+  </si>
+  <si>
+    <t>T1_Security</t>
+  </si>
+  <si>
+    <t>T1_CBP</t>
+  </si>
+  <si>
+    <t>T1_Lounge</t>
+  </si>
+  <si>
+    <t>T1_Boarding</t>
+  </si>
+  <si>
+    <t>T1_Immigration</t>
+  </si>
+  <si>
+    <t>T1_Baggage</t>
+  </si>
+  <si>
+    <t>T2_Checkin</t>
+  </si>
+  <si>
+    <t>T2_Security</t>
+  </si>
+  <si>
+    <t>T2_CBP</t>
+  </si>
+  <si>
+    <t>T2_Lounge</t>
+  </si>
+  <si>
+    <t>T2_Boarding</t>
+  </si>
+  <si>
+    <t>T2_Immigration</t>
+  </si>
+  <si>
+    <t>T2_Baggage</t>
   </si>
 </sst>
 </file>
@@ -389,25 +392,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -451,48 +454,48 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="B2">
-        <v>100</v>
+        <v>450</v>
       </c>
       <c r="C2">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="D2">
+        <v>500</v>
+      </c>
+      <c r="E2">
+        <v>300</v>
+      </c>
+      <c r="F2">
         <v>150</v>
       </c>
-      <c r="E2">
+      <c r="G2">
+        <v>500</v>
+      </c>
+      <c r="H2">
         <v>150</v>
       </c>
-      <c r="F2">
-        <v>100</v>
-      </c>
-      <c r="G2">
+      <c r="I2">
+        <v>450</v>
+      </c>
+      <c r="J2">
+        <v>150</v>
+      </c>
+      <c r="K2">
+        <v>500</v>
+      </c>
+      <c r="L2">
         <v>300</v>
       </c>
-      <c r="H2">
-        <v>50</v>
-      </c>
-      <c r="I2">
-        <v>100</v>
-      </c>
-      <c r="J2">
-        <v>100</v>
-      </c>
-      <c r="K2">
+      <c r="M2">
         <v>150</v>
       </c>
-      <c r="L2">
-        <v>150</v>
-      </c>
-      <c r="M2">
-        <v>100</v>
-      </c>
       <c r="N2">
-        <v>300</v>
+        <v>500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Intraday Staff reallocation and Config sorted
</commit_message>
<xml_diff>
--- a/data/PAX Config.xlsx
+++ b/data/PAX Config.xlsx
@@ -1,93 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6070f6eab8483c11/Desktop/DAA/live/DAA-Project/data/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="11_F25DC773A252ABDACC104835C91E41EE5ADE58E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{876FFA43-5221-40C9-AB91-598849D0A682}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="162913" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
-  <si>
-    <t>T1_Checkin</t>
-  </si>
-  <si>
-    <t>T1_Security</t>
-  </si>
-  <si>
-    <t>T1_CBP</t>
-  </si>
-  <si>
-    <t>T1_Lounge</t>
-  </si>
-  <si>
-    <t>T1_Boarding</t>
-  </si>
-  <si>
-    <t>T1_Immigration</t>
-  </si>
-  <si>
-    <t>T1_Baggage</t>
-  </si>
-  <si>
-    <t>T2_Checkin</t>
-  </si>
-  <si>
-    <t>T2_Security</t>
-  </si>
-  <si>
-    <t>T2_CBP</t>
-  </si>
-  <si>
-    <t>T2_Lounge</t>
-  </si>
-  <si>
-    <t>T2_Boarding</t>
-  </si>
-  <si>
-    <t>T2_Immigration</t>
-  </si>
-  <si>
-    <t>T2_Baggage</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -106,26 +46,81 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -390,111 +385,143 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.140625" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col width="13.140625" customWidth="1" min="1" max="1"/>
+    <col width="10.28515625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="9.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="11.140625" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="13.85546875" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="10.7109375" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="10.140625" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="10.28515625" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="6.85546875" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="9.42578125" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="11.140625" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="13.85546875" bestFit="1" customWidth="1" min="13" max="13"/>
+    <col width="10.7109375" bestFit="1" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" t="s">
-        <v>13</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>T1_Checkin</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>T1_Security</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>T1_CBP</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>T1_Lounge</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>T1_Boarding</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>T1_Immigration</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>T1_Baggage</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>T2_Checkin</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>T2_Security</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>T2_CBP</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>T2_Lounge</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>T2_Boarding</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>T2_Immigration</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>T2_Baggage</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2">
+    <row r="2">
+      <c r="A2" t="n">
         <v>150</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="n">
         <v>450</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>150</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>500</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="n">
         <v>300</v>
       </c>
-      <c r="F2">
+      <c r="F2" t="n">
         <v>150</v>
       </c>
-      <c r="G2">
+      <c r="G2" t="n">
         <v>500</v>
       </c>
-      <c r="H2">
+      <c r="H2" t="n">
         <v>150</v>
       </c>
-      <c r="I2">
+      <c r="I2" t="n">
         <v>450</v>
       </c>
-      <c r="J2">
+      <c r="J2" t="n">
         <v>150</v>
       </c>
-      <c r="K2">
+      <c r="K2" t="n">
         <v>500</v>
       </c>
-      <c r="L2">
+      <c r="L2" t="n">
         <v>300</v>
       </c>
-      <c r="M2">
+      <c r="M2" t="n">
         <v>150</v>
       </c>
-      <c r="N2">
+      <c r="N2" t="n">
         <v>500</v>
       </c>
     </row>

</xml_diff>